<commit_message>
Synchronize Excel database and main.py to GitHub
</commit_message>
<xml_diff>
--- a/AI_Stock_Investment_Dashboard.xlsx
+++ b/AI_Stock_Investment_Dashboard.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="168" formatCode="\+#,##0.0;\-#,##0.0;0.0"/>
     <numFmt numFmtId="169" formatCode="+#,##0.0;-#,##0.0;0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +96,12 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="FF196F3D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00196F3D"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -221,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -377,6 +383,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -819,13 +831,13 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1827.67</v>
+        <v>1867.21</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>-0.26</v>
+        <v>7.2</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>-0.0001</v>
+        <v>0.0039</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>854000000</v>
@@ -846,13 +858,13 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1966.77</v>
+        <v>2013.35</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>-1.81</v>
+        <v>17.64</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>-0.0009</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>210000000</v>
@@ -873,13 +885,13 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>333.06</v>
+        <v>313.16</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>-0.13</v>
+        <v>0</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>68000000</v>
@@ -900,13 +912,13 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>127.5</v>
+        <v>129.97</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>1.12</v>
+        <v>-0.3</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.008699999999999999</v>
+        <v>-0.0023</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>42000000</v>
@@ -927,13 +939,13 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1961.04</v>
-      </c>
-      <c r="C11" s="49" t="n">
-        <v>0.78</v>
+        <v>2014</v>
+      </c>
+      <c r="C11" s="57" t="n">
+        <v>16.4</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.0004</v>
+        <v>0.008199999999999999</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>254000</v>
@@ -983,7 +995,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
@@ -1007,12 +1019,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Thấp - Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Chưa cần hạ tỷ trọng danh mục vội vàng</t>
+          <t>Hạ tỷ trọng đòn bẩy (margin), phòng thủ danh mục</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1039,12 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Tập trung giải ngân vào các nhóm ngành dẫn dắt dòng tiền</t>
+          <t>Cơ hội giải ngân ít, nên kiên nhẫn quan sát điểm cân bằng</t>
         </is>
       </c>
     </row>
@@ -1087,10 +1099,10 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1961.04</v>
+        <v>2014</v>
       </c>
       <c r="C22" s="40" t="n">
-        <v>-5.730000000000018</v>
+        <v>0.6500000000000909</v>
       </c>
       <c r="D22" s="41" t="inlineStr">
         <is>
@@ -1102,11 +1114,11 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>1,971 - 1,976</t>
+          <t>2,024 - 2,029 điểm</t>
         </is>
       </c>
       <c r="G22" s="8" t="n">
-        <v>1953</v>
+        <v>2006</v>
       </c>
     </row>
   </sheetData>
@@ -1229,7 +1241,7 @@
         <v>4100</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>71600</v>
+        <v>73200</v>
       </c>
       <c r="F7" s="8">
         <f>C7*D7</f>
@@ -1270,7 +1282,7 @@
         <v>3800</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>25310</v>
+        <v>25750</v>
       </c>
       <c r="F8" s="8">
         <f>C8*D8</f>
@@ -1311,7 +1323,7 @@
         <v>800</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>20670</v>
+        <v>22300</v>
       </c>
       <c r="F9" s="8">
         <f>C9*D9</f>
@@ -1352,7 +1364,7 @@
         <v>79000</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>4750</v>
+        <v>4590</v>
       </c>
       <c r="F10" s="8">
         <f>C10*D10</f>
@@ -2401,70 +2413,70 @@
     <row r="7" ht="20.1" customHeight="1" s="51">
       <c r="A7" s="42" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="B7" s="52" t="n">
-        <v>-327.6</v>
-      </c>
-      <c r="C7" s="52" t="n">
-        <v>-2.5</v>
+        <v>-166.8</v>
+      </c>
+      <c r="C7" s="53" t="n">
+        <v>90.59999999999999</v>
       </c>
       <c r="D7" s="53" t="n">
-        <v>332.1</v>
+        <v>69.3</v>
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>Khối ngoại bán ròng mạnh gây áp lực tâm lý chốt lời lên toàn bộ thị trường.</t>
+          <t>Lực cầu chủ động từ dòng tiền lớn gia tăng tại các nhóm ngành dẫn dắt dòng tiền.</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H7" s="54" t="inlineStr">
         <is>
-          <t>Tăng mạnh</t>
+          <t>Tăng nhẹ</t>
         </is>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.92</v>
+        <v>0.75</v>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>1,865 - 1,889 điểm</t>
+          <t>1,860 - 1,885 điểm</t>
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr">
         <is>
-          <t>Kỹ thuật: Chỉ số giữ vững trên SMA20, MACD duy trì phân kỳ dương ủng hộ động lực tăng điểm ngắn hạn. Vĩ mô QT: Bối cảnh thị trường quốc tế (Dow Jones, Châu Á) giao dịch ổn định, giảm thiểu rủi ro biến động liên thông. Chính sách: Tỷ giá USD/VND chịu áp lực lớn buộc SBV duy trì nghiệp vụ hút tiền qua thị trường mở (OMO) để cân bằng lãi suất.</t>
+          <t>Kỹ thuật: VN-Index tích lũy chặt chẽ quanh 1,867.22 (hỗ trợ cứng 1,850 - 1,860, kháng cự mạnh 1,880 - 1,900) với lực cầu tốt. Tác động ngoại: S&amp;P 500 ở mức 7,467.44 điểm, tâm lý dòng tiền nội thận trọng theo dõi báo cáo lao động Mỹ ngày 02/07. Vĩ mô VN: Mùa BCTC Q2 và bán niên khởi động tạo sự phân hóa; dòng tiền nội ưu tiên các cổ phiếu đầu ngành như FPT, MBB, SSI.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20.1" customHeight="1" s="51">
       <c r="A8" s="42" t="inlineStr">
         <is>
-          <t>24/06/2026</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="B8" s="52" t="n">
-        <v>-219.3</v>
+        <v>-152.2</v>
       </c>
       <c r="C8" s="53" t="n">
-        <v>56.9</v>
+        <v>65</v>
       </c>
       <c r="D8" s="53" t="n">
-        <v>154.9</v>
+        <v>79.2</v>
       </c>
       <c r="E8" s="45" t="inlineStr">
         <is>
-          <t>Lực cầu chủ động từ dòng tiền lớn gia tăng tại các nhóm ngành dẫn dắt dòng tiền.</t>
+          <t>Dòng tiền lớn tiếp tục mua ròng nhóm Công nghệ và Ngân hàng hỗ trợ thị trường nâng đỡ chỉ số.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="H8" s="54" t="inlineStr">
@@ -2473,42 +2485,42 @@
         </is>
       </c>
       <c r="I8" s="39" t="n">
-        <v>0.88</v>
+        <v>0.71</v>
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>1,870 - 1,894 điểm</t>
+          <t>1,865 - 1,890 điểm</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>Chính sách: Tỷ giá USD/VND chịu áp lực lớn buộc SBV duy trì nghiệp vụ hút tiền qua thị trường mở (OMO) để cân bằng lãi suất. Kỹ thuật: Chỉ số giữ vững trên SMA20, MACD duy trì phân kỳ dương ủng hộ động lực tăng điểm ngắn hạn. Vĩ mô QT: Bối cảnh thị trường quốc tế (Dow Jones, Châu Á) giao dịch ổn định, giảm thiểu rủi ro biến động liên thông.</t>
+          <t>Kỹ thuật: Chỉ số thử thách kháng cự 1,880 - 1,900 điểm, đòi hỏi thanh khoản cải thiện và lực mua lan rộng ngoài nhóm trụ. Tác động ngoại: Áp lực tỷ giá USD/VND (25,450 VND) kích hoạt tâm lý phòng thủ ngắn hạn của khối ngoại. Vĩ mô VN: Tiến trình nâng hạng thị trường lên mới nổi FTSE tiếp tục là động lực trung hạn thu hút sự chú ý của dòng vốn FII.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20.1" customHeight="1" s="51">
       <c r="A9" s="42" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="B9" s="52" t="n">
-        <v>-193.2</v>
+        <v>-166.8</v>
       </c>
       <c r="C9" s="53" t="n">
-        <v>80.7</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="D9" s="53" t="n">
-        <v>109</v>
+        <v>69.3</v>
       </c>
       <c r="E9" s="45" t="inlineStr">
         <is>
-          <t>Dòng tiền lớn tiếp tục mua ròng nhóm Công nghệ và Ngân hàng hỗ trợ thị trường nâng đỡ chỉ số.</t>
+          <t>Lực cầu chủ động từ dòng tiền lớn gia tăng tại các nhóm ngành dẫn dắt dòng tiền.</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="H9" s="55" t="inlineStr">
@@ -2517,104 +2529,104 @@
         </is>
       </c>
       <c r="I9" s="39" t="n">
-        <v>0.84</v>
+        <v>0.67</v>
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>1,871 - 1,893 điểm</t>
+          <t>1,866 - 1,889 điểm</t>
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>Vĩ mô QT: Bối cảnh thị trường quốc tế (Dow Jones, Châu Á) giao dịch ổn định, giảm thiểu rủi ro biến động liên thông. Chính sách: Tỷ giá USD/VND chịu áp lực lớn buộc SBV duy trì nghiệp vụ hút tiền qua thị trường mở (OMO) để cân bằng lãi suất. Kỹ thuật: VN-Index đi ngang biên độ hẹp quanh hỗ trợ SMA20, thanh khoản tích lũy chờ dòng tiền bứt phá.</t>
+          <t>Kỹ thuật: Hỗ trợ gần 1,850 - 1,860 điểm được củng cố tốt nhờ lực cầu nội chủ động đỡ giá ở các nhịp rung lắc kỹ thuật. Tác động ngoại: Theo dõi sát sao chỉ số CPI Mỹ ngày 14/07 và PPI ngày 15/07 để đánh giá áp lực lên tỷ giá trong nước. Vĩ mô VN: Kỳ vọng giải ngân vốn đầu tư công tăng tốc và gỡ vướng pháp lý BĐS là điểm tựa vững chắc cho tâm lý thị trường.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20.1" customHeight="1" s="51">
       <c r="A10" s="42" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="B10" s="52" t="n">
-        <v>-227.4</v>
+        <v>-155.8</v>
       </c>
       <c r="C10" s="53" t="n">
-        <v>79.09999999999999</v>
+        <v>100.1</v>
       </c>
       <c r="D10" s="53" t="n">
-        <v>150.2</v>
+        <v>64.3</v>
       </c>
       <c r="E10" s="45" t="inlineStr">
         <is>
-          <t>Dòng tiền lớn hoạt động tích cực ở nhóm Thép và Bất động sản giúp luân phiên bùng nổ.</t>
+          <t>Lực cầu chủ động từ dòng tiền lớn gia tăng tại các nhóm ngành dẫn dắt dòng tiền.</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="H10" s="54" t="inlineStr">
-        <is>
-          <t>Tăng nhẹ</t>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="H10" s="56" t="inlineStr">
+        <is>
+          <t>Giảm nhẹ</t>
         </is>
       </c>
       <c r="I10" s="39" t="n">
-        <v>0.8</v>
+        <v>0.63</v>
       </c>
       <c r="J10" s="9" t="inlineStr">
         <is>
-          <t>1,875 - 1,900 điểm</t>
+          <t>1,860 - 1,884 điểm</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>Kỹ thuật: VN-Index thử thách kênh hỗ trợ trung hạn SMA50. Vĩ mô QT: Bối cảnh thị trường quốc tế (Dow Jones, Châu Á) giao dịch ổn định, giảm thiểu rủi ro biến động liên thông. Chính sách: Tỷ giá USD/VND chịu áp lực lớn buộc SBV duy trì nghiệp vụ hút tiền qua thị trường mở (OMO) để cân bằng lãi suất.</t>
+          <t>Kỹ thuật: VN-Index thử thách đường SMA50 trung hạn, thanh khoản cạn kiệt mở ra cơ hội tích lũy cổ phiếu giá trị giá tốt. Tác động ngoại: Bối cảnh tài chính quốc tế ổn định giúp giảm thiểu đáng kể rủi ro biến động liên thông đối với thị trường cơ sở. Vĩ mô VN: CPI được kiểm soát tốt và GDP tăng trưởng vững chắc giúp SBV giữ vững lập trường chính sách tiền tệ nới lỏng linh hoạt.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20.1" customHeight="1" s="51">
       <c r="A11" s="42" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>29/06/2026</t>
         </is>
       </c>
       <c r="B11" s="52" t="n">
-        <v>-416.1</v>
-      </c>
-      <c r="C11" s="52" t="n">
-        <v>-42.1</v>
+        <v>-446.4</v>
+      </c>
+      <c r="C11" s="53" t="n">
+        <v>1.1</v>
       </c>
       <c r="D11" s="53" t="n">
-        <v>459.2</v>
+        <v>437.5</v>
       </c>
       <c r="E11" s="45" t="inlineStr">
         <is>
-          <t>Áp lực bán ròng gia tăng ở nhóm ngành tài chính, dòng tiền dịch chuyển sang phòng thủ.</t>
+          <t>Khối ngoại bán ròng mạnh gây áp lực tâm lý chốt lời lên toàn bộ thị trường.</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="H11" s="54" t="inlineStr">
         <is>
-          <t>Tăng mạnh</t>
+          <t>Tăng nhẹ</t>
         </is>
       </c>
       <c r="I11" s="39" t="n">
-        <v>0.76</v>
+        <v>0.59</v>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>1,890 - 1,915 điểm</t>
+          <t>1,865 - 1,890 điểm</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>Kỹ thuật: Chỉ số giữ vững trên SMA20, MACD duy trì phân kỳ dương ủng hộ động lực tăng điểm ngắn hạn. Vĩ mô QT: Bối cảnh thị trường quốc tế (Dow Jones, Châu Á) giao dịch ổn định, giảm thiểu rủi ro biến động liên thông. Chính sách: Kỳ vọng SBV nới lỏng nhẹ thanh khoản hệ thống khi áp lực tỷ giá hạ nhiệt vào cuối chu kỳ.</t>
+          <t>Kỹ thuật: Cơ hội bứt phá biên tích lũy để hướng tới kiểm định đỉnh lịch sử cũ 1,936.55 điểm khi lực cầu cải thiện rõ rệt. Tác động ngoại: Tâm lý thận trọng bao trùm trước thềm cuộc họp Fed ngày 29/07 và công bố PCE ngày 30/07. Vĩ mô VN: Kết quả tăng trưởng lợi nhuận ấn tượng của các nhóm ngành trụ cột sẽ là động cơ chính dẫn dắt chỉ số đi lên.</t>
         </is>
       </c>
     </row>

</xml_diff>